<commit_message>
fix: update WhatsApp number to 9045651385, fix code formatting
</commit_message>
<xml_diff>
--- a/warranty_registry_backup.xlsx
+++ b/warranty_registry_backup.xlsx
@@ -507,6 +507,11 @@
           <t>2026-06-23 12:15:57</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>